<commit_message>
T2275_ July 21 2024 changes
</commit_message>
<xml_diff>
--- a/TestData/LV_T2274_VerifyValidationRulesOnEventExpense.xlsx
+++ b/TestData/LV_T2274_VerifyValidationRulesOnEventExpense.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F573FB0-19D4-4CB8-A04E-DBF86CE80E45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30D17814-9AD9-4407-85FF-C8903F72FA14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="43">
   <si>
     <t>StdUser</t>
   </si>
@@ -122,9 +122,6 @@
   </si>
   <si>
     <t>FVATestOpportunity</t>
-  </si>
-  <si>
-    <t>Sonika Goyal</t>
   </si>
   <si>
     <t>App Name</t>
@@ -156,6 +153,12 @@
   </si>
   <si>
     <t>Automation Test Event</t>
+  </si>
+  <si>
+    <t>Please fill out the required fields: Number of guests is Required. Please select at least one Team Member.</t>
+  </si>
+  <si>
+    <t>Vijay Kumar</t>
   </si>
 </sst>
 </file>
@@ -529,12 +532,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -552,12 +555,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -633,7 +636,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:15" s="2" customFormat="1" ht="72" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" s="2" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>28</v>
       </c>
@@ -641,7 +644,7 @@
         <v>5</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>7</v>
+        <v>41</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>27</v>
@@ -650,7 +653,7 @@
         <v>9</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>14</v>
@@ -677,7 +680,7 @@
         <v>30</v>
       </c>
       <c r="O2" s="2" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -743,10 +746,10 @@
         <v>25</v>
       </c>
       <c r="P1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q1" s="1" t="s">
         <v>35</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:17" s="2" customFormat="1" ht="72" x14ac:dyDescent="0.3">
@@ -793,13 +796,13 @@
         <v>30</v>
       </c>
       <c r="O2" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="P2" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="P2" s="3" t="s">
+      <c r="Q2" s="3" t="s">
         <v>38</v>
-      </c>
-      <c r="Q2" s="3" t="s">
-        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>